<commit_message>
Spec moteur/organique : source unique V_MOTEUR_CAL + elasticite en membre calcule
Les onglets Le moteur et Budget de marque pointent desormais une source
unique (V_MOTEUR_CAL, grain campus x exercice) au lieu du melange
V_CAMPAGNES + socle. L'elasticite est documentee comme membre calcule
Tagetik (LN[2026]/LN[2024]) et non plus comme colonne de vue.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/RESTITUTIONS_EDUSERVICES.xlsx
+++ b/eduservices/tagetik/RESTITUTIONS_EDUSERVICES.xlsx
@@ -1270,7 +1270,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3678,7 +3678,7 @@
       </c>
       <c r="B59" s="60" t="inlineStr">
         <is>
-          <t>V_CAMPAGNES (calibration : élasticité acquisition, conversion, réfs)  +  socle AW_002_000002_000001 (CA/inscrit réel)</t>
+          <t>V_MOTEUR_CAL  (source unique : séries annuelles par campus × exercice)</t>
         </is>
       </c>
     </row>
@@ -3690,7 +3690,7 @@
       </c>
       <c r="B60" s="60" t="inlineStr">
         <is>
-          <t>ENTITY (campus) ▸ groupé par MARQUE   —   l'élasticité vit au campus, la marque = sous-total</t>
+          <t>ENTITY (campus) ▸ groupé par MARQUE   en lignes   ·   EXERCICE (2024·2025·2026) en colonnes</t>
         </is>
       </c>
     </row>
@@ -3726,75 +3726,87 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="59" t="inlineStr">
+      <c r="A64" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   EXERCICE</t>
+        </is>
+      </c>
+      <c r="B64" s="63" t="inlineStr">
+        <is>
+          <t>2024 · 2025 · 2026   (réel ; le budget = 2027)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="59" t="inlineStr">
         <is>
           <t>Champs de la vue</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Leads payants (L.pay 24/25/26)</t>
-        </is>
-      </c>
-      <c r="B65" s="63" t="inlineStr">
-        <is>
-          <t>PAID_REF / LEAD_REF  (V_CAMPAGNES)</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="64" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Budget acquisition (Bud.24/25/26)</t>
+          <t xml:space="preserve">   Leads payants (L.pay 24/25/26)</t>
         </is>
       </c>
       <c r="B66" s="63" t="inlineStr">
         <is>
-          <t>SPEND_ACQ_REF  (compte 6231, V_CAMPAGNES)</t>
+          <t>LEAD_PAY  (par EXERCICE)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="64" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Élasticité</t>
+          <t xml:space="preserve">   Budget acquisition (Bud.24/25/26)</t>
         </is>
       </c>
       <c r="B67" s="63" t="inlineStr">
         <is>
-          <t>REND_ACQ = régression 3 ans  =SLOPE(LN(leads);LN(budget))</t>
+          <t>SPEND_ACQ  (compte 6231, par EXERCICE)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="64" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Conversion</t>
+          <t xml:space="preserve">   Élasticité</t>
         </is>
       </c>
       <c r="B68" s="63" t="inlineStr">
         <is>
-          <t>CONVERSION = inscrits ÷ leads  (V_CAMPAGNES)</t>
+          <t>MEMBRE CALCULÉ = LN(LEAD_PAY[2026]/LEAD_PAY[2024]) ÷ LN(SPEND_ACQ[2026]/SPEND_ACQ[2024])</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="64" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Conversion</t>
+        </is>
+      </c>
+      <c r="B69" s="63" t="inlineStr">
+        <is>
+          <t>CONVERSION = INSCRITS ÷ LEAD_TOT  (par EXERCICE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="64" t="inlineStr">
+        <is>
           <t xml:space="preserve">   CA / inscrit</t>
         </is>
       </c>
-      <c r="B69" s="63" t="inlineStr">
-        <is>
-          <t>(VOL_NEW·REV_STUD + VOL_NEW·REV_FRAIS_INS) ÷ VOL_NEW  par campus (socle 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="65" t="n"/>
-      <c r="B70" s="65" t="n"/>
+      <c r="B70" s="63" t="inlineStr">
+        <is>
+          <t>CA_PAR_INSCRIT  (par campus × EXERCICE, vrai chiffre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="65" t="n"/>
+      <c r="B71" s="65" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3807,7 +3819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5011,7 +5023,7 @@
       </c>
       <c r="B49" s="60" t="inlineStr">
         <is>
-          <t>V_CAMPAGNES (élasticité marque, réfs organiques)  +  socle AW_002_000002_000001</t>
+          <t>V_MOTEUR_CAL  (source unique : séries annuelles par campus × exercice)</t>
         </is>
       </c>
     </row>
@@ -5023,7 +5035,7 @@
       </c>
       <c r="B50" s="60" t="inlineStr">
         <is>
-          <t>ENTITY (campus) ▸ groupé par MARQUE</t>
+          <t>ENTITY (campus) ▸ groupé par MARQUE   en lignes   ·   EXERCICE (2024·2025·2026) en colonnes</t>
         </is>
       </c>
     </row>
@@ -5059,51 +5071,63 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="59" t="inlineStr">
+      <c r="A54" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   EXERCICE</t>
+        </is>
+      </c>
+      <c r="B54" s="63" t="inlineStr">
+        <is>
+          <t>2024 · 2025 · 2026   (réel ; le budget = 2027)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="59" t="inlineStr">
         <is>
           <t>Champs de la vue</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Budget de marque (Bud.mq 24/25/26)</t>
-        </is>
-      </c>
-      <c r="B55" s="63" t="inlineStr">
-        <is>
-          <t>SPEND_BRAND_REF  (compte 6236, V_CAMPAGNES)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="64" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Leads organiques (Org.24/25/26)</t>
+          <t xml:space="preserve">   Budget de marque (Bud.mq 24/25/26)</t>
         </is>
       </c>
       <c r="B56" s="63" t="inlineStr">
         <is>
-          <t>ORG_REF  (V_CAMPAGNES)</t>
+          <t>SPEND_BRAND  (compte 6236, par EXERCICE)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="64" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Leads organiques (Org.24/25/26)</t>
+        </is>
+      </c>
+      <c r="B57" s="63" t="inlineStr">
+        <is>
+          <t>LEAD_ORG  (par EXERCICE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="64" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Élasticité marque</t>
         </is>
       </c>
-      <c r="B57" s="63" t="inlineStr">
-        <is>
-          <t>REND_BRAND = régression 3 ans  =SLOPE(LN(organiques);LN(budget marque))</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="65" t="n"/>
-      <c r="B58" s="65" t="n"/>
+      <c r="B58" s="63" t="inlineStr">
+        <is>
+          <t>MEMBRE CALCULÉ = LN(LEAD_ORG[2026]/LEAD_ORG[2024]) ÷ LN(SPEND_BRAND[2026]/SPEND_BRAND[2024])</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="65" t="n"/>
+      <c r="B59" s="65" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>